<commit_message>
research(agent-architecture): clarification/elicitation 컴포넌트 추가 + 블로그 인덱스 등재
- 블로그 3.6절 신설: Clarification/Elicitation(되묻기) — Claude Code AskUserQuestion(네이티브),
  MCP elicitation / A2A input-required(프로토콜), Codex 자율지향 부재, 모델 ask-rate 튜닝.
  clarification/approval/interrupt 3분법 정리.
- index.md AI Agent & Systems 섹션에 리서치 등재(GitHub Pages 노출).
- PPT Slide 20 추가 및 번호 재정렬, 참고문헌 XLSX 2건 추가(62건).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D1iCQPSFN3sYBzAG5z5Z87
</commit_message>
<xml_diff>
--- a/2026-07-24-agent-architecture/agent-architecture-references.xlsx
+++ b/2026-07-24-agent-architecture/agent-architecture-references.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2596,6 +2596,76 @@
       <c r="G61" s="2" t="inlineStr">
         <is>
           <t>L8 상용</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Handle approvals and user input</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic (Claude Code / Agent SDK docs)</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>https://code.claude.com/docs/en/agent-sdk/user-input</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>clarification(AskUserQuestion, 옵션 자동생성 + 모달 + 루프 블록)과 approval(권한 게이팅)을 명시적으로 분리. 사용자 입력/승인 처리.</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>L3 clarification</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>MCP elicitation: Request user input at runtime</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>WorkOS</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>https://workos.com/blog/mcp-elicitation</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>2025~2026</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>MCP Elicitation(elicitation/create, ElicitationRequest): 서버가 실행 중 사용자 입력을 요청. 2026 로드맵 stateless(InputRequiredResult) 재설계.</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>L3 clarification</t>
         </is>
       </c>
     </row>
@@ -2661,6 +2731,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>